<commit_message>
Power islands and vias placement, only we re missing diodes models
</commit_message>
<xml_diff>
--- a/BOM_TFG_v1.xlsx
+++ b/BOM_TFG_v1.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Effer\Desktop\TFG_PCB\TFG_Ultrawideband_pulse_generator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F9DEBD9F-F48F-4520-A8CD-2823349BB18F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B7F0B95-F696-4CB1-86DE-55D0BFFD63E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4755" yWindow="675" windowWidth="17610" windowHeight="13155" xr2:uid="{B80083CD-1C1E-41D5-BE04-2C929030B1F4}"/>
   </bookViews>
   <sheets>
-    <sheet name="rs" sheetId="2" r:id="rId1"/>
+    <sheet name="mouser" sheetId="2" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="39">
   <si>
     <t>Distribuidor</t>
   </si>
@@ -69,18 +69,9 @@
     <t>Inversor TTL</t>
   </si>
   <si>
-    <t>MC74VHC1GT14DBVT1G</t>
-  </si>
-  <si>
-    <t>863-MC74VHC1GT14DBVG</t>
-  </si>
-  <si>
     <t>MOUSER</t>
   </si>
   <si>
-    <t>Inersor TTL  de 1 canal MC74VHC1GT14DBVT1G</t>
-  </si>
-  <si>
     <t>https://www.mouser.es/ProductDetail/Vishay-Sfernice/TS53YL105MR10?qs=MsRaK5qBadQL4ESplrFiTw%3D%3D</t>
   </si>
   <si>
@@ -114,26 +105,6 @@
     <t>https://www.mouser.es/ProductDetail/Infineon-Technologies/BFP-420-H6433?qs=9Vqdt%252BdHmfLTU8JasfSKRw%3D%3D</t>
   </si>
   <si>
-    <t>https://www.mouser.es/ProductDetail/onsemi/MC74VHC1GT14DBVT1G?qs=vLWxofP3U2y98PQgYBav%252Bw%3D%3D</t>
-  </si>
-  <si>
-    <t>LDO de 12V a 5V AMS1117-5.0</t>
-  </si>
-  <si>
-    <t>DIGIKEY</t>
-  </si>
-  <si>
-    <t>https://www.digikey.es/es/products/detail/evvo/AMS1117-5-0/24370130</t>
-  </si>
-  <si>
-    <t>AMS1117-5.0</t>
-  </si>
-  <si>
-    <t>5272-AMS1117-5.0TR-ND - Cinta y rollo (TR)
-5272-AMS1117-5.0CT-ND - Cinta cortada (CT)
-5272-AMS1117-5.0DKR-ND - Digi-Reel®</t>
-  </si>
-  <si>
     <t>Transistor NPN de potencia media y encapsulado SOT 23 -- BFR 35AP E6327</t>
   </si>
   <si>
@@ -147,6 +118,30 @@
   </si>
   <si>
     <t>PENDIENTE</t>
+  </si>
+  <si>
+    <t>LDO de 12V a 5V TS1117BCW50 RPG</t>
+  </si>
+  <si>
+    <t>TS1117BCW50 RPG</t>
+  </si>
+  <si>
+    <t>821-TS1117BCW50RPG</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Taiwan-Semiconductor/TS1117BCW50-RPG?qs=5aG0NVq1C4ylI5XQUTRxrQ%3D%3D</t>
+  </si>
+  <si>
+    <t>Inersor TTL  de 1 canal  MC74VHC1GT04DFT2G</t>
+  </si>
+  <si>
+    <t>MC74VHC1GT04DFT2G</t>
+  </si>
+  <si>
+    <t>863-C74VHC1GT04DFT2G</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/onsemi/MC74VHC1GT04DFT2G?qs=1tjIq5M9V4PBMtfRHM%2Fd7w%3D%3D</t>
   </si>
 </sst>
 </file>
@@ -159,7 +154,7 @@
     <numFmt numFmtId="166" formatCode="#,##0.00\ &quot;€&quot;"/>
     <numFmt numFmtId="167" formatCode="_-* #,##0.00\ _€_-;\-* #,##0.00\ _€_-;_-* &quot;-&quot;??\ _€_-;_-@_-"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -196,12 +191,6 @@
     <font>
       <sz val="12"/>
       <color rgb="FF333333"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color rgb="FF444444"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -290,7 +279,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="167" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
@@ -343,15 +332,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -372,86 +356,64 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="2" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="4" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -773,7 +735,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{592B7D0C-4226-432C-B929-B07F2B31A9DC}">
-  <dimension ref="A1:N27"/>
+  <dimension ref="A1:M25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -785,7 +747,7 @@
     <col min="10" max="10" width="29.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -817,18 +779,18 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:14" s="11" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" s="11" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="C2" s="19" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="D2" s="19" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="E2" s="6"/>
       <c r="F2" s="7">
@@ -837,24 +799,24 @@
       <c r="G2" s="7"/>
       <c r="H2" s="8"/>
       <c r="I2" s="9" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="J2" s="10" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:14" s="11" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" s="11" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="E3" s="6"/>
       <c r="F3" s="7">
@@ -863,24 +825,24 @@
       <c r="G3" s="7"/>
       <c r="H3" s="8"/>
       <c r="I3" s="9" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="J3" s="10" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B4" s="16" t="s">
         <v>12</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4" s="19" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E4" s="13"/>
       <c r="F4" s="14">
@@ -889,24 +851,24 @@
       <c r="G4" s="14"/>
       <c r="H4" s="13"/>
       <c r="I4" s="15" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="J4" s="17" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="120" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="B5" s="16" t="s">
-        <v>30</v>
-      </c>
-      <c r="C5" s="20" t="s">
+      <c r="C5" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="D5" s="19" t="s">
         <v>33</v>
-      </c>
-      <c r="D5" s="21" t="s">
-        <v>34</v>
       </c>
       <c r="E5" s="13"/>
       <c r="F5" s="14">
@@ -915,383 +877,287 @@
       <c r="G5" s="14"/>
       <c r="H5" s="13"/>
       <c r="I5" s="15" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="J5" s="17" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="K5" s="18"/>
       <c r="L5" s="18"/>
       <c r="M5" s="18"/>
     </row>
-    <row r="6" spans="1:14" ht="30" x14ac:dyDescent="0.25">
-      <c r="A6" s="25" t="s">
-        <v>16</v>
-      </c>
-      <c r="B6" s="26" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="25" t="s">
+    <row r="6" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" s="22" t="s">
         <v>14</v>
       </c>
+      <c r="B6" s="23" t="s">
+        <v>35</v>
+      </c>
+      <c r="C6" s="19" t="s">
+        <v>36</v>
+      </c>
       <c r="D6" s="19" t="s">
-        <v>15</v>
-      </c>
-      <c r="E6" s="27"/>
-      <c r="F6" s="28">
+        <v>37</v>
+      </c>
+      <c r="E6" s="24"/>
+      <c r="F6" s="25">
         <v>20</v>
       </c>
-      <c r="G6" s="28"/>
-      <c r="H6" s="27"/>
-      <c r="I6" s="29" t="s">
-        <v>29</v>
-      </c>
-      <c r="J6" s="30" t="s">
+      <c r="G6" s="25"/>
+      <c r="H6" s="24"/>
+      <c r="I6" s="26" t="s">
+        <v>38</v>
+      </c>
+      <c r="J6" s="27" t="s">
         <v>13</v>
       </c>
       <c r="K6" s="18"/>
       <c r="L6" s="18"/>
       <c r="M6" s="18"/>
     </row>
-    <row r="7" spans="1:14" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="33" t="s">
-        <v>39</v>
-      </c>
-      <c r="B7" s="34" t="s">
-        <v>37</v>
-      </c>
-      <c r="C7" s="33"/>
-      <c r="D7" s="33"/>
-      <c r="E7" s="35"/>
-      <c r="F7" s="35"/>
-      <c r="G7" s="35"/>
-      <c r="H7" s="36"/>
-      <c r="I7" s="37"/>
-      <c r="J7" s="38"/>
-      <c r="K7" s="39"/>
-      <c r="L7" s="39"/>
-      <c r="M7" s="39"/>
-      <c r="N7" s="40"/>
-    </row>
-    <row r="8" spans="1:14" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="33" t="s">
-        <v>39</v>
-      </c>
-      <c r="B8" s="41" t="s">
-        <v>38</v>
-      </c>
-      <c r="C8" s="33"/>
-      <c r="D8" s="33"/>
-      <c r="E8" s="35"/>
-      <c r="F8" s="35"/>
-      <c r="G8" s="35"/>
-      <c r="H8" s="36"/>
-      <c r="I8" s="37"/>
-      <c r="J8" s="38"/>
-      <c r="K8" s="39"/>
-      <c r="L8" s="39"/>
-      <c r="M8" s="39"/>
-      <c r="N8" s="40"/>
-    </row>
-    <row r="9" spans="1:14" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="42"/>
-      <c r="B9" s="43"/>
-      <c r="C9" s="42"/>
-      <c r="D9" s="42"/>
-      <c r="E9" s="44"/>
-      <c r="F9" s="44"/>
-      <c r="G9" s="44"/>
-      <c r="H9" s="45"/>
-      <c r="I9" s="37"/>
-      <c r="J9" s="46"/>
-      <c r="K9" s="47"/>
-      <c r="L9" s="47"/>
-      <c r="M9" s="47"/>
-      <c r="N9" s="40"/>
-    </row>
-    <row r="10" spans="1:14" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="42"/>
-      <c r="B10" s="48"/>
-      <c r="C10" s="42"/>
-      <c r="D10" s="49"/>
-      <c r="E10" s="44"/>
-      <c r="F10" s="44"/>
-      <c r="G10" s="44"/>
-      <c r="H10" s="45"/>
-      <c r="I10" s="37"/>
-      <c r="J10" s="46"/>
-      <c r="K10" s="47"/>
-      <c r="L10" s="47"/>
-      <c r="M10" s="47"/>
-      <c r="N10" s="40"/>
-    </row>
-    <row r="11" spans="1:14" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="42"/>
-      <c r="B11" s="48"/>
-      <c r="C11" s="42"/>
-      <c r="D11" s="42"/>
-      <c r="E11" s="50"/>
-      <c r="F11" s="51"/>
-      <c r="G11" s="51"/>
-      <c r="H11" s="50"/>
-      <c r="I11" s="37"/>
-      <c r="J11" s="46"/>
-      <c r="K11" s="47"/>
-      <c r="L11" s="47"/>
-      <c r="M11" s="47"/>
-      <c r="N11" s="40"/>
-    </row>
-    <row r="12" spans="1:14" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="42"/>
-      <c r="B12" s="46"/>
-      <c r="C12" s="52"/>
-      <c r="D12" s="53"/>
-      <c r="E12" s="45"/>
-      <c r="F12" s="54"/>
-      <c r="G12" s="55"/>
-      <c r="H12" s="56"/>
-      <c r="I12" s="37"/>
-      <c r="J12" s="46"/>
-      <c r="K12" s="47"/>
-      <c r="L12" s="47"/>
-      <c r="M12" s="47"/>
-      <c r="N12" s="40"/>
-    </row>
-    <row r="13" spans="1:14" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="42"/>
-      <c r="B13" s="57"/>
-      <c r="C13" s="52"/>
-      <c r="D13" s="53"/>
-      <c r="E13" s="45"/>
-      <c r="F13" s="54"/>
-      <c r="G13" s="55"/>
-      <c r="H13" s="56"/>
-      <c r="I13" s="37"/>
-      <c r="J13" s="46"/>
-      <c r="K13" s="47"/>
-      <c r="L13" s="47"/>
-      <c r="M13" s="47"/>
-      <c r="N13" s="40"/>
-    </row>
-    <row r="14" spans="1:14" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="42"/>
-      <c r="B14" s="57"/>
-      <c r="C14" s="52"/>
-      <c r="D14" s="53"/>
-      <c r="E14" s="45"/>
-      <c r="F14" s="54"/>
-      <c r="G14" s="55"/>
-      <c r="H14" s="56"/>
-      <c r="I14" s="58"/>
-      <c r="J14" s="46"/>
-      <c r="K14" s="49"/>
-      <c r="L14" s="42"/>
-      <c r="M14" s="42"/>
-      <c r="N14" s="40"/>
-    </row>
-    <row r="15" spans="1:14" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="42"/>
-      <c r="B15" s="57"/>
-      <c r="C15" s="52"/>
-      <c r="D15" s="53"/>
-      <c r="E15" s="45"/>
-      <c r="F15" s="54"/>
-      <c r="G15" s="55"/>
-      <c r="H15" s="45"/>
-      <c r="I15" s="58"/>
-      <c r="J15" s="57"/>
-      <c r="K15" s="42"/>
-      <c r="L15" s="42"/>
-      <c r="M15" s="42"/>
-      <c r="N15" s="40"/>
-    </row>
-    <row r="16" spans="1:14" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="42"/>
-      <c r="B16" s="57"/>
-      <c r="C16" s="52"/>
-      <c r="D16" s="53"/>
-      <c r="E16" s="45"/>
-      <c r="F16" s="54"/>
-      <c r="G16" s="55"/>
-      <c r="H16" s="45"/>
-      <c r="I16" s="58"/>
-      <c r="J16" s="57"/>
-      <c r="K16" s="42"/>
-      <c r="L16" s="42"/>
-      <c r="M16" s="42"/>
-      <c r="N16" s="40"/>
-    </row>
-    <row r="17" spans="1:14" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="42"/>
-      <c r="B17" s="57"/>
-      <c r="C17" s="52"/>
-      <c r="D17" s="53"/>
-      <c r="E17" s="45"/>
-      <c r="F17" s="54"/>
-      <c r="G17" s="55"/>
-      <c r="H17" s="56"/>
-      <c r="I17" s="58"/>
-      <c r="J17" s="46"/>
-      <c r="K17" s="42"/>
-      <c r="L17" s="42"/>
-      <c r="M17" s="42"/>
-      <c r="N17" s="40"/>
-    </row>
-    <row r="18" spans="1:14" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="42"/>
-      <c r="B18" s="57"/>
-      <c r="C18" s="52"/>
-      <c r="D18" s="53"/>
-      <c r="E18" s="45"/>
-      <c r="F18" s="54"/>
-      <c r="G18" s="55"/>
-      <c r="H18" s="56"/>
-      <c r="I18" s="58"/>
-      <c r="J18" s="46"/>
-      <c r="K18" s="42"/>
-      <c r="L18" s="42"/>
-      <c r="M18" s="42"/>
-      <c r="N18" s="40"/>
-    </row>
-    <row r="19" spans="1:14" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="42"/>
-      <c r="B19" s="57"/>
-      <c r="C19" s="52"/>
-      <c r="D19" s="53"/>
-      <c r="E19" s="45"/>
-      <c r="F19" s="54"/>
-      <c r="G19" s="55"/>
-      <c r="H19" s="56"/>
-      <c r="I19" s="58"/>
-      <c r="J19" s="46"/>
-      <c r="K19" s="42"/>
-      <c r="L19" s="42"/>
-      <c r="M19" s="42"/>
-      <c r="N19" s="40"/>
-    </row>
-    <row r="20" spans="1:14" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="42"/>
-      <c r="B20" s="57"/>
-      <c r="C20" s="52"/>
-      <c r="D20" s="53"/>
-      <c r="E20" s="45"/>
-      <c r="F20" s="54"/>
-      <c r="G20" s="55"/>
-      <c r="H20" s="56"/>
-      <c r="I20" s="37"/>
-      <c r="J20" s="46"/>
-      <c r="K20" s="47"/>
-      <c r="L20" s="47"/>
-      <c r="M20" s="47"/>
-      <c r="N20" s="40"/>
-    </row>
-    <row r="21" spans="1:14" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="42"/>
-      <c r="B21" s="57"/>
-      <c r="C21" s="52"/>
-      <c r="D21" s="53"/>
-      <c r="E21" s="45"/>
-      <c r="F21" s="54"/>
-      <c r="G21" s="55"/>
-      <c r="H21" s="56"/>
-      <c r="I21" s="37"/>
-      <c r="J21" s="46"/>
-      <c r="K21" s="47"/>
-      <c r="L21" s="47"/>
-      <c r="M21" s="47"/>
-      <c r="N21" s="40"/>
-    </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A22" s="47"/>
-      <c r="B22" s="47"/>
-      <c r="C22" s="47"/>
-      <c r="D22" s="47"/>
-      <c r="E22" s="47"/>
-      <c r="F22" s="47"/>
-      <c r="G22" s="47"/>
-      <c r="H22" s="47"/>
-      <c r="I22" s="47"/>
-      <c r="J22" s="47"/>
-      <c r="K22" s="47"/>
-      <c r="L22" s="47"/>
-      <c r="M22" s="47"/>
-      <c r="N22" s="59"/>
-    </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A23" s="60"/>
-      <c r="B23" s="47"/>
-      <c r="C23" s="47"/>
-      <c r="D23" s="47"/>
-      <c r="E23" s="47"/>
-      <c r="F23" s="47"/>
-      <c r="G23" s="47"/>
-      <c r="H23" s="47"/>
-      <c r="I23" s="47"/>
-      <c r="J23" s="47"/>
-      <c r="K23" s="47"/>
-      <c r="L23" s="47"/>
-      <c r="M23" s="47"/>
-      <c r="N23" s="59"/>
-    </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A24" s="31"/>
-      <c r="B24" s="32"/>
-      <c r="C24" s="22"/>
-      <c r="D24" s="22"/>
-      <c r="E24" s="22"/>
-      <c r="F24" s="22"/>
-      <c r="G24" s="22"/>
-      <c r="H24" s="22"/>
-      <c r="I24" s="22"/>
-      <c r="J24" s="22"/>
-      <c r="K24" s="22"/>
-      <c r="L24" s="22"/>
-      <c r="M24" s="22"/>
-    </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A25" s="23"/>
-      <c r="B25" s="24"/>
-      <c r="C25" s="22"/>
-      <c r="D25" s="22"/>
-      <c r="E25" s="22"/>
-      <c r="F25" s="22"/>
-      <c r="G25" s="22"/>
-      <c r="H25" s="22"/>
-      <c r="I25" s="22"/>
-      <c r="J25" s="22"/>
-      <c r="K25" s="22"/>
-      <c r="L25" s="22"/>
-      <c r="M25" s="22"/>
-    </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A26" s="22"/>
-      <c r="B26" s="22"/>
-      <c r="C26" s="22"/>
-      <c r="D26" s="22"/>
-      <c r="E26" s="22"/>
-      <c r="F26" s="22"/>
-      <c r="G26" s="22"/>
-      <c r="H26" s="22"/>
-      <c r="I26" s="22"/>
-      <c r="J26" s="22"/>
-      <c r="K26" s="22"/>
-      <c r="L26" s="22"/>
-      <c r="M26" s="22"/>
-    </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A27" s="22"/>
-      <c r="B27" s="22"/>
-      <c r="C27" s="22"/>
-      <c r="D27" s="22"/>
-      <c r="E27" s="22"/>
-      <c r="F27" s="22"/>
-      <c r="G27" s="22"/>
-      <c r="H27" s="22"/>
-      <c r="I27" s="22"/>
-      <c r="J27" s="22"/>
-      <c r="K27" s="22"/>
-      <c r="L27" s="22"/>
-      <c r="M27" s="22"/>
+    <row r="7" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="30" t="s">
+        <v>30</v>
+      </c>
+      <c r="B7" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" s="30"/>
+      <c r="D7" s="30"/>
+      <c r="E7" s="32"/>
+      <c r="F7" s="32"/>
+      <c r="G7" s="32"/>
+      <c r="H7" s="33"/>
+      <c r="I7" s="34"/>
+      <c r="J7" s="35"/>
+      <c r="K7" s="18"/>
+      <c r="L7" s="18"/>
+      <c r="M7" s="18"/>
+    </row>
+    <row r="8" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="30" t="s">
+        <v>30</v>
+      </c>
+      <c r="B8" s="36" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" s="30"/>
+      <c r="D8" s="30"/>
+      <c r="E8" s="32"/>
+      <c r="F8" s="32"/>
+      <c r="G8" s="32"/>
+      <c r="H8" s="33"/>
+      <c r="I8" s="34"/>
+      <c r="J8" s="35"/>
+      <c r="K8" s="18"/>
+      <c r="L8" s="18"/>
+      <c r="M8" s="18"/>
+    </row>
+    <row r="9" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="30"/>
+      <c r="B9" s="36"/>
+      <c r="C9" s="30"/>
+      <c r="D9" s="30"/>
+      <c r="E9" s="32"/>
+      <c r="F9" s="32"/>
+      <c r="G9" s="32"/>
+      <c r="H9" s="33"/>
+      <c r="I9" s="34"/>
+      <c r="J9" s="35"/>
+      <c r="K9"/>
+      <c r="L9"/>
+      <c r="M9"/>
+    </row>
+    <row r="10" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="30"/>
+      <c r="B10" s="31"/>
+      <c r="C10" s="30"/>
+      <c r="D10" s="37"/>
+      <c r="E10" s="32"/>
+      <c r="F10" s="32"/>
+      <c r="G10" s="32"/>
+      <c r="H10" s="33"/>
+      <c r="I10" s="34"/>
+      <c r="J10" s="35"/>
+      <c r="K10"/>
+      <c r="L10"/>
+      <c r="M10"/>
+    </row>
+    <row r="11" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="30"/>
+      <c r="B11" s="31"/>
+      <c r="C11" s="30"/>
+      <c r="D11" s="30"/>
+      <c r="E11" s="38"/>
+      <c r="F11" s="39"/>
+      <c r="G11" s="39"/>
+      <c r="H11" s="38"/>
+      <c r="I11" s="34"/>
+      <c r="J11" s="35"/>
+      <c r="K11"/>
+      <c r="L11"/>
+      <c r="M11"/>
+    </row>
+    <row r="12" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="30"/>
+      <c r="B12" s="35"/>
+      <c r="C12" s="40"/>
+      <c r="D12" s="41"/>
+      <c r="E12" s="33"/>
+      <c r="F12" s="42"/>
+      <c r="G12" s="43"/>
+      <c r="H12" s="44"/>
+      <c r="I12" s="34"/>
+      <c r="J12" s="35"/>
+      <c r="K12"/>
+      <c r="L12"/>
+      <c r="M12"/>
+    </row>
+    <row r="13" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="30"/>
+      <c r="B13" s="45"/>
+      <c r="C13" s="40"/>
+      <c r="D13" s="41"/>
+      <c r="E13" s="33"/>
+      <c r="F13" s="42"/>
+      <c r="G13" s="43"/>
+      <c r="H13" s="44"/>
+      <c r="I13" s="34"/>
+      <c r="J13" s="35"/>
+      <c r="K13"/>
+      <c r="L13"/>
+      <c r="M13"/>
+    </row>
+    <row r="14" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="30"/>
+      <c r="B14" s="45"/>
+      <c r="C14" s="40"/>
+      <c r="D14" s="41"/>
+      <c r="E14" s="33"/>
+      <c r="F14" s="42"/>
+      <c r="G14" s="43"/>
+      <c r="H14" s="44"/>
+      <c r="I14" s="46"/>
+      <c r="J14" s="35"/>
+      <c r="K14" s="37"/>
+      <c r="L14" s="30"/>
+      <c r="M14" s="30"/>
+    </row>
+    <row r="15" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="30"/>
+      <c r="B15" s="45"/>
+      <c r="C15" s="40"/>
+      <c r="D15" s="41"/>
+      <c r="E15" s="33"/>
+      <c r="F15" s="42"/>
+      <c r="G15" s="43"/>
+      <c r="H15" s="33"/>
+      <c r="I15" s="46"/>
+      <c r="J15" s="45"/>
+      <c r="K15" s="30"/>
+      <c r="L15" s="30"/>
+      <c r="M15" s="30"/>
+    </row>
+    <row r="16" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="30"/>
+      <c r="B16" s="45"/>
+      <c r="C16" s="40"/>
+      <c r="D16" s="41"/>
+      <c r="E16" s="33"/>
+      <c r="F16" s="42"/>
+      <c r="G16" s="43"/>
+      <c r="H16" s="33"/>
+      <c r="I16" s="46"/>
+      <c r="J16" s="45"/>
+      <c r="K16" s="30"/>
+      <c r="L16" s="30"/>
+      <c r="M16" s="30"/>
+    </row>
+    <row r="17" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="30"/>
+      <c r="B17" s="45"/>
+      <c r="C17" s="40"/>
+      <c r="D17" s="41"/>
+      <c r="E17" s="33"/>
+      <c r="F17" s="42"/>
+      <c r="G17" s="43"/>
+      <c r="H17" s="44"/>
+      <c r="I17" s="46"/>
+      <c r="J17" s="35"/>
+      <c r="K17" s="30"/>
+      <c r="L17" s="30"/>
+      <c r="M17" s="30"/>
+    </row>
+    <row r="18" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="30"/>
+      <c r="B18" s="45"/>
+      <c r="C18" s="40"/>
+      <c r="D18" s="41"/>
+      <c r="E18" s="33"/>
+      <c r="F18" s="42"/>
+      <c r="G18" s="43"/>
+      <c r="H18" s="44"/>
+      <c r="I18" s="46"/>
+      <c r="J18" s="35"/>
+      <c r="K18" s="30"/>
+      <c r="L18" s="30"/>
+      <c r="M18" s="30"/>
+    </row>
+    <row r="19" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="30"/>
+      <c r="B19" s="45"/>
+      <c r="C19" s="40"/>
+      <c r="D19" s="41"/>
+      <c r="E19" s="33"/>
+      <c r="F19" s="42"/>
+      <c r="G19" s="43"/>
+      <c r="H19" s="44"/>
+      <c r="I19" s="46"/>
+      <c r="J19" s="35"/>
+      <c r="K19" s="30"/>
+      <c r="L19" s="30"/>
+      <c r="M19" s="30"/>
+    </row>
+    <row r="20" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="30"/>
+      <c r="B20" s="45"/>
+      <c r="C20" s="40"/>
+      <c r="D20" s="41"/>
+      <c r="E20" s="33"/>
+      <c r="F20" s="42"/>
+      <c r="G20" s="43"/>
+      <c r="H20" s="44"/>
+      <c r="I20" s="34"/>
+      <c r="J20" s="35"/>
+      <c r="K20"/>
+      <c r="L20"/>
+      <c r="M20"/>
+    </row>
+    <row r="21" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="30"/>
+      <c r="B21" s="45"/>
+      <c r="C21" s="40"/>
+      <c r="D21" s="41"/>
+      <c r="E21" s="33"/>
+      <c r="F21" s="42"/>
+      <c r="G21" s="43"/>
+      <c r="H21" s="44"/>
+      <c r="I21" s="34"/>
+      <c r="J21" s="35"/>
+      <c r="K21"/>
+      <c r="L21"/>
+      <c r="M21"/>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A23" s="47"/>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A24" s="28"/>
+      <c r="B24" s="29"/>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A25" s="20"/>
+      <c r="B25" s="21"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Updated Schottky and SRD diodes in PCB and BOM, everything is ready to check, only DRC is missing
</commit_message>
<xml_diff>
--- a/BOM_TFG_v1.xlsx
+++ b/BOM_TFG_v1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Effer\Desktop\TFG_PCB\TFG_Ultrawideband_pulse_generator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B7F0B95-F696-4CB1-86DE-55D0BFFD63E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAF7E0F4-3AE0-419D-8226-A45604A785CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4755" yWindow="675" windowWidth="17610" windowHeight="13155" xr2:uid="{B80083CD-1C1E-41D5-BE04-2C929030B1F4}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="46">
   <si>
     <t>Distribuidor</t>
   </si>
@@ -111,15 +111,6 @@
     <t>LDO de 12V a 5V</t>
   </si>
   <si>
-    <t>SRD</t>
-  </si>
-  <si>
-    <t>SCHOTTKY</t>
-  </si>
-  <si>
-    <t>PENDIENTE</t>
-  </si>
-  <si>
     <t>LDO de 12V a 5V TS1117BCW50 RPG</t>
   </si>
   <si>
@@ -142,6 +133,36 @@
   </si>
   <si>
     <t>https://www.mouser.es/ProductDetail/onsemi/MC74VHC1GT04DFT2G?qs=1tjIq5M9V4PBMtfRHM%2Fd7w%3D%3D</t>
+  </si>
+  <si>
+    <t>873-SMS3923-079LF</t>
+  </si>
+  <si>
+    <t>SMS3923-079LF</t>
+  </si>
+  <si>
+    <t>SCHOTTKY -  SMS3923-079LF</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Skyworks-Solutions-Inc/SMS3923-079LF?qs=VAD5mMsctQDWkZ8Ev6tpzg%3D%3D</t>
+  </si>
+  <si>
+    <t>SRD - MA144769-287T</t>
+  </si>
+  <si>
+    <t>MA144769-287T</t>
+  </si>
+  <si>
+    <t>937-MA144769-287T</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/MACOM/MA144769-287T?qs=xL%2FyUNPmvLYcaIK%2F6M7KHA%3D%3D</t>
+  </si>
+  <si>
+    <t>Diode SRD</t>
+  </si>
+  <si>
+    <t>Diode Schottky</t>
   </si>
 </sst>
 </file>
@@ -195,7 +216,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -211,12 +232,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -330,7 +345,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -350,9 +364,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -415,6 +426,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -786,10 +801,10 @@
       <c r="B2" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C2" s="19" t="s">
+      <c r="C2" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="D2" s="19" t="s">
+      <c r="D2" s="18" t="s">
         <v>23</v>
       </c>
       <c r="E2" s="6"/>
@@ -841,7 +856,7 @@
       <c r="C4" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="D4" s="19" t="s">
+      <c r="D4" s="18" t="s">
         <v>17</v>
       </c>
       <c r="E4" s="13"/>
@@ -862,13 +877,13 @@
         <v>14</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>31</v>
-      </c>
-      <c r="C5" s="19" t="s">
-        <v>32</v>
-      </c>
-      <c r="D5" s="19" t="s">
-        <v>33</v>
+        <v>28</v>
+      </c>
+      <c r="C5" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="D5" s="18" t="s">
+        <v>30</v>
       </c>
       <c r="E5" s="13"/>
       <c r="F5" s="14">
@@ -877,290 +892,313 @@
       <c r="G5" s="14"/>
       <c r="H5" s="13"/>
       <c r="I5" s="15" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="J5" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="K5" s="18"/>
-      <c r="L5" s="18"/>
-      <c r="M5" s="18"/>
+      <c r="K5" s="46"/>
+      <c r="L5" s="46"/>
+      <c r="M5" s="46"/>
     </row>
     <row r="6" spans="1:13" ht="30" x14ac:dyDescent="0.25">
-      <c r="A6" s="22" t="s">
+      <c r="A6" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="23" t="s">
+      <c r="B6" s="22" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="D6" s="18" t="s">
+        <v>34</v>
+      </c>
+      <c r="E6" s="23"/>
+      <c r="F6" s="24">
+        <v>20</v>
+      </c>
+      <c r="G6" s="24"/>
+      <c r="H6" s="23"/>
+      <c r="I6" s="47" t="s">
         <v>35</v>
       </c>
-      <c r="C6" s="19" t="s">
+      <c r="J6" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="K6" s="46"/>
+      <c r="L6" s="46"/>
+      <c r="M6" s="46"/>
+    </row>
+    <row r="7" spans="1:13" s="11" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A7" s="28" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="29" t="s">
+        <v>40</v>
+      </c>
+      <c r="C7" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="D7" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="E7" s="30"/>
+      <c r="F7" s="30">
+        <v>20</v>
+      </c>
+      <c r="G7" s="30"/>
+      <c r="H7" s="31"/>
+      <c r="I7" s="32" t="s">
+        <v>43</v>
+      </c>
+      <c r="J7" s="33" t="s">
+        <v>44</v>
+      </c>
+      <c r="K7" s="46"/>
+      <c r="L7" s="46"/>
+      <c r="M7" s="46"/>
+    </row>
+    <row r="8" spans="1:13" s="11" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A8" s="28" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="34" t="s">
+        <v>38</v>
+      </c>
+      <c r="C8" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="D8" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="D6" s="19" t="s">
-        <v>37</v>
-      </c>
-      <c r="E6" s="24"/>
-      <c r="F6" s="25">
-        <v>20</v>
-      </c>
-      <c r="G6" s="25"/>
-      <c r="H6" s="24"/>
-      <c r="I6" s="26" t="s">
-        <v>38</v>
-      </c>
-      <c r="J6" s="27" t="s">
-        <v>13</v>
-      </c>
-      <c r="K6" s="18"/>
-      <c r="L6" s="18"/>
-      <c r="M6" s="18"/>
-    </row>
-    <row r="7" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="30" t="s">
-        <v>30</v>
-      </c>
-      <c r="B7" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="C7" s="30"/>
-      <c r="D7" s="30"/>
-      <c r="E7" s="32"/>
-      <c r="F7" s="32"/>
-      <c r="G7" s="32"/>
-      <c r="H7" s="33"/>
-      <c r="I7" s="34"/>
-      <c r="J7" s="35"/>
-      <c r="K7" s="18"/>
-      <c r="L7" s="18"/>
-      <c r="M7" s="18"/>
-    </row>
-    <row r="8" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="30" t="s">
-        <v>30</v>
-      </c>
-      <c r="B8" s="36" t="s">
-        <v>29</v>
-      </c>
-      <c r="C8" s="30"/>
-      <c r="D8" s="30"/>
-      <c r="E8" s="32"/>
-      <c r="F8" s="32"/>
-      <c r="G8" s="32"/>
-      <c r="H8" s="33"/>
-      <c r="I8" s="34"/>
-      <c r="J8" s="35"/>
-      <c r="K8" s="18"/>
-      <c r="L8" s="18"/>
-      <c r="M8" s="18"/>
-    </row>
-    <row r="9" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="30"/>
-      <c r="B9" s="36"/>
-      <c r="C9" s="30"/>
-      <c r="D9" s="30"/>
-      <c r="E9" s="32"/>
-      <c r="F9" s="32"/>
-      <c r="G9" s="32"/>
-      <c r="H9" s="33"/>
-      <c r="I9" s="34"/>
-      <c r="J9" s="35"/>
+      <c r="E8" s="30"/>
+      <c r="F8" s="30">
+        <v>40</v>
+      </c>
+      <c r="G8" s="30"/>
+      <c r="H8" s="31"/>
+      <c r="I8" s="32" t="s">
+        <v>39</v>
+      </c>
+      <c r="J8" s="33" t="s">
+        <v>45</v>
+      </c>
+      <c r="K8" s="46"/>
+      <c r="L8" s="46"/>
+      <c r="M8" s="46"/>
+    </row>
+    <row r="9" spans="1:13" s="11" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A9" s="28"/>
+      <c r="B9" s="34"/>
+      <c r="C9" s="18"/>
+      <c r="D9" s="18"/>
+      <c r="E9" s="30"/>
+      <c r="F9" s="30"/>
+      <c r="G9" s="30"/>
+      <c r="H9" s="31"/>
+      <c r="I9" s="32"/>
+      <c r="J9" s="33"/>
       <c r="K9"/>
       <c r="L9"/>
       <c r="M9"/>
     </row>
     <row r="10" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="30"/>
-      <c r="B10" s="31"/>
-      <c r="C10" s="30"/>
-      <c r="D10" s="37"/>
-      <c r="E10" s="32"/>
-      <c r="F10" s="32"/>
-      <c r="G10" s="32"/>
-      <c r="H10" s="33"/>
-      <c r="I10" s="34"/>
-      <c r="J10" s="35"/>
+      <c r="A10" s="28"/>
+      <c r="B10" s="29"/>
+      <c r="C10" s="28"/>
+      <c r="D10" s="35"/>
+      <c r="E10" s="30"/>
+      <c r="F10" s="30"/>
+      <c r="G10" s="30"/>
+      <c r="H10" s="31"/>
+      <c r="I10" s="32"/>
+      <c r="J10" s="33"/>
       <c r="K10"/>
       <c r="L10"/>
       <c r="M10"/>
     </row>
     <row r="11" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="30"/>
-      <c r="B11" s="31"/>
-      <c r="C11" s="30"/>
-      <c r="D11" s="30"/>
-      <c r="E11" s="38"/>
-      <c r="F11" s="39"/>
-      <c r="G11" s="39"/>
-      <c r="H11" s="38"/>
-      <c r="I11" s="34"/>
-      <c r="J11" s="35"/>
+      <c r="A11" s="28"/>
+      <c r="B11" s="29"/>
+      <c r="C11" s="28"/>
+      <c r="D11" s="28"/>
+      <c r="E11" s="36"/>
+      <c r="F11" s="37"/>
+      <c r="G11" s="37"/>
+      <c r="H11" s="36"/>
+      <c r="I11" s="32"/>
+      <c r="J11" s="33"/>
       <c r="K11"/>
       <c r="L11"/>
       <c r="M11"/>
     </row>
     <row r="12" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="30"/>
-      <c r="B12" s="35"/>
-      <c r="C12" s="40"/>
-      <c r="D12" s="41"/>
-      <c r="E12" s="33"/>
-      <c r="F12" s="42"/>
-      <c r="G12" s="43"/>
-      <c r="H12" s="44"/>
-      <c r="I12" s="34"/>
-      <c r="J12" s="35"/>
+      <c r="A12" s="28"/>
+      <c r="B12" s="33"/>
+      <c r="C12" s="38"/>
+      <c r="D12" s="39"/>
+      <c r="E12" s="31"/>
+      <c r="F12" s="40"/>
+      <c r="G12" s="41"/>
+      <c r="H12" s="42"/>
+      <c r="I12" s="32"/>
+      <c r="J12" s="33"/>
       <c r="K12"/>
       <c r="L12"/>
       <c r="M12"/>
     </row>
     <row r="13" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="30"/>
-      <c r="B13" s="45"/>
-      <c r="C13" s="40"/>
-      <c r="D13" s="41"/>
-      <c r="E13" s="33"/>
-      <c r="F13" s="42"/>
-      <c r="G13" s="43"/>
-      <c r="H13" s="44"/>
-      <c r="I13" s="34"/>
-      <c r="J13" s="35"/>
+      <c r="A13" s="28"/>
+      <c r="B13" s="43"/>
+      <c r="C13" s="38"/>
+      <c r="D13" s="39"/>
+      <c r="E13" s="31"/>
+      <c r="F13" s="40"/>
+      <c r="G13" s="41"/>
+      <c r="H13" s="42"/>
+      <c r="I13" s="32"/>
+      <c r="J13" s="33"/>
       <c r="K13"/>
       <c r="L13"/>
       <c r="M13"/>
     </row>
     <row r="14" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="30"/>
-      <c r="B14" s="45"/>
-      <c r="C14" s="40"/>
-      <c r="D14" s="41"/>
-      <c r="E14" s="33"/>
-      <c r="F14" s="42"/>
-      <c r="G14" s="43"/>
-      <c r="H14" s="44"/>
-      <c r="I14" s="46"/>
-      <c r="J14" s="35"/>
-      <c r="K14" s="37"/>
-      <c r="L14" s="30"/>
-      <c r="M14" s="30"/>
+      <c r="A14" s="28"/>
+      <c r="B14" s="43"/>
+      <c r="C14" s="38"/>
+      <c r="D14" s="39"/>
+      <c r="E14" s="31"/>
+      <c r="F14" s="40"/>
+      <c r="G14" s="41"/>
+      <c r="H14" s="42"/>
+      <c r="I14" s="44"/>
+      <c r="J14" s="33"/>
+      <c r="K14" s="35"/>
+      <c r="L14" s="28"/>
+      <c r="M14" s="28"/>
     </row>
     <row r="15" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="30"/>
-      <c r="B15" s="45"/>
-      <c r="C15" s="40"/>
-      <c r="D15" s="41"/>
-      <c r="E15" s="33"/>
-      <c r="F15" s="42"/>
-      <c r="G15" s="43"/>
-      <c r="H15" s="33"/>
-      <c r="I15" s="46"/>
-      <c r="J15" s="45"/>
-      <c r="K15" s="30"/>
-      <c r="L15" s="30"/>
-      <c r="M15" s="30"/>
+      <c r="A15" s="28"/>
+      <c r="B15" s="43"/>
+      <c r="C15" s="38"/>
+      <c r="D15" s="39"/>
+      <c r="E15" s="31"/>
+      <c r="F15" s="40"/>
+      <c r="G15" s="41"/>
+      <c r="H15" s="31"/>
+      <c r="I15" s="44"/>
+      <c r="J15" s="43"/>
+      <c r="K15" s="28"/>
+      <c r="L15" s="28"/>
+      <c r="M15" s="28"/>
     </row>
     <row r="16" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="30"/>
-      <c r="B16" s="45"/>
-      <c r="C16" s="40"/>
-      <c r="D16" s="41"/>
-      <c r="E16" s="33"/>
-      <c r="F16" s="42"/>
-      <c r="G16" s="43"/>
-      <c r="H16" s="33"/>
-      <c r="I16" s="46"/>
-      <c r="J16" s="45"/>
-      <c r="K16" s="30"/>
-      <c r="L16" s="30"/>
-      <c r="M16" s="30"/>
+      <c r="A16" s="28"/>
+      <c r="B16" s="43"/>
+      <c r="C16" s="38"/>
+      <c r="D16" s="39"/>
+      <c r="E16" s="31"/>
+      <c r="F16" s="40"/>
+      <c r="G16" s="41"/>
+      <c r="H16" s="31"/>
+      <c r="I16" s="44"/>
+      <c r="J16" s="43"/>
+      <c r="K16" s="28"/>
+      <c r="L16" s="28"/>
+      <c r="M16" s="28"/>
     </row>
     <row r="17" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="30"/>
-      <c r="B17" s="45"/>
-      <c r="C17" s="40"/>
-      <c r="D17" s="41"/>
-      <c r="E17" s="33"/>
-      <c r="F17" s="42"/>
-      <c r="G17" s="43"/>
-      <c r="H17" s="44"/>
-      <c r="I17" s="46"/>
-      <c r="J17" s="35"/>
-      <c r="K17" s="30"/>
-      <c r="L17" s="30"/>
-      <c r="M17" s="30"/>
+      <c r="A17" s="28"/>
+      <c r="B17" s="43"/>
+      <c r="C17" s="38"/>
+      <c r="D17" s="39"/>
+      <c r="E17" s="31"/>
+      <c r="F17" s="40"/>
+      <c r="G17" s="41"/>
+      <c r="H17" s="42"/>
+      <c r="I17" s="44"/>
+      <c r="J17" s="33"/>
+      <c r="K17" s="28"/>
+      <c r="L17" s="28"/>
+      <c r="M17" s="28"/>
     </row>
     <row r="18" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="30"/>
-      <c r="B18" s="45"/>
-      <c r="C18" s="40"/>
-      <c r="D18" s="41"/>
-      <c r="E18" s="33"/>
-      <c r="F18" s="42"/>
-      <c r="G18" s="43"/>
-      <c r="H18" s="44"/>
-      <c r="I18" s="46"/>
-      <c r="J18" s="35"/>
-      <c r="K18" s="30"/>
-      <c r="L18" s="30"/>
-      <c r="M18" s="30"/>
+      <c r="A18" s="28"/>
+      <c r="B18" s="43"/>
+      <c r="C18" s="38"/>
+      <c r="D18" s="39"/>
+      <c r="E18" s="31"/>
+      <c r="F18" s="40"/>
+      <c r="G18" s="41"/>
+      <c r="H18" s="42"/>
+      <c r="I18" s="44"/>
+      <c r="J18" s="33"/>
+      <c r="K18" s="28"/>
+      <c r="L18" s="28"/>
+      <c r="M18" s="28"/>
     </row>
     <row r="19" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="30"/>
-      <c r="B19" s="45"/>
-      <c r="C19" s="40"/>
-      <c r="D19" s="41"/>
-      <c r="E19" s="33"/>
-      <c r="F19" s="42"/>
-      <c r="G19" s="43"/>
-      <c r="H19" s="44"/>
-      <c r="I19" s="46"/>
-      <c r="J19" s="35"/>
-      <c r="K19" s="30"/>
-      <c r="L19" s="30"/>
-      <c r="M19" s="30"/>
+      <c r="A19" s="28"/>
+      <c r="B19" s="43"/>
+      <c r="C19" s="38"/>
+      <c r="D19" s="39"/>
+      <c r="E19" s="31"/>
+      <c r="F19" s="40"/>
+      <c r="G19" s="41"/>
+      <c r="H19" s="42"/>
+      <c r="I19" s="44"/>
+      <c r="J19" s="33"/>
+      <c r="K19" s="28"/>
+      <c r="L19" s="28"/>
+      <c r="M19" s="28"/>
     </row>
     <row r="20" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="30"/>
-      <c r="B20" s="45"/>
-      <c r="C20" s="40"/>
-      <c r="D20" s="41"/>
-      <c r="E20" s="33"/>
-      <c r="F20" s="42"/>
-      <c r="G20" s="43"/>
-      <c r="H20" s="44"/>
-      <c r="I20" s="34"/>
-      <c r="J20" s="35"/>
+      <c r="A20" s="28"/>
+      <c r="B20" s="43"/>
+      <c r="C20" s="38"/>
+      <c r="D20" s="39"/>
+      <c r="E20" s="31"/>
+      <c r="F20" s="40"/>
+      <c r="G20" s="41"/>
+      <c r="H20" s="42"/>
+      <c r="I20" s="32"/>
+      <c r="J20" s="33"/>
       <c r="K20"/>
       <c r="L20"/>
       <c r="M20"/>
     </row>
     <row r="21" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="30"/>
-      <c r="B21" s="45"/>
-      <c r="C21" s="40"/>
-      <c r="D21" s="41"/>
-      <c r="E21" s="33"/>
-      <c r="F21" s="42"/>
-      <c r="G21" s="43"/>
-      <c r="H21" s="44"/>
-      <c r="I21" s="34"/>
-      <c r="J21" s="35"/>
+      <c r="A21" s="28"/>
+      <c r="B21" s="43"/>
+      <c r="C21" s="38"/>
+      <c r="D21" s="39"/>
+      <c r="E21" s="31"/>
+      <c r="F21" s="40"/>
+      <c r="G21" s="41"/>
+      <c r="H21" s="42"/>
+      <c r="I21" s="32"/>
+      <c r="J21" s="33"/>
       <c r="K21"/>
       <c r="L21"/>
       <c r="M21"/>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A23" s="47"/>
+      <c r="A23" s="45"/>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A24" s="28"/>
-      <c r="B24" s="29"/>
+      <c r="A24" s="26"/>
+      <c r="B24" s="27"/>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A25" s="20"/>
-      <c r="B25" s="21"/>
+      <c r="A25" s="19"/>
+      <c r="B25" s="20"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="I6" r:id="rId1" xr:uid="{38C36DE8-EDB6-461D-8534-EB0F1250A34D}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Uploaded datasheet for main components
</commit_message>
<xml_diff>
--- a/BOM_TFG_v1.xlsx
+++ b/BOM_TFG_v1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Effer\Desktop\TFG_PCB\TFG_Ultrawideband_pulse_generator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAF7E0F4-3AE0-419D-8226-A45604A785CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03920204-11C0-4BAC-8F4B-7D986C637F8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4755" yWindow="675" windowWidth="17610" windowHeight="13155" xr2:uid="{B80083CD-1C1E-41D5-BE04-2C929030B1F4}"/>
   </bookViews>
@@ -294,7 +294,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="167" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
@@ -320,9 +320,6 @@
     <xf numFmtId="165" fontId="3" fillId="3" borderId="2" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -427,8 +424,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -794,17 +793,17 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:13" s="11" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" s="10" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>14</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="D2" s="17" t="s">
         <v>23</v>
       </c>
       <c r="E2" s="6"/>
@@ -813,14 +812,14 @@
       </c>
       <c r="G2" s="7"/>
       <c r="H2" s="8"/>
-      <c r="I2" s="9" t="s">
+      <c r="I2" s="46" t="s">
         <v>24</v>
       </c>
-      <c r="J2" s="10" t="s">
+      <c r="J2" s="9" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:13" s="11" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" s="10" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>14</v>
       </c>
@@ -839,10 +838,10 @@
       </c>
       <c r="G3" s="7"/>
       <c r="H3" s="8"/>
-      <c r="I3" s="9" t="s">
+      <c r="I3" s="46" t="s">
         <v>25</v>
       </c>
-      <c r="J3" s="10" t="s">
+      <c r="J3" s="9" t="s">
         <v>21</v>
       </c>
     </row>
@@ -850,355 +849,352 @@
       <c r="A4" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="16" t="s">
+      <c r="B4" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="C4" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="D4" s="18" t="s">
+      <c r="D4" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="E4" s="13"/>
-      <c r="F4" s="14">
+      <c r="E4" s="12"/>
+      <c r="F4" s="13">
         <v>40</v>
       </c>
-      <c r="G4" s="14"/>
-      <c r="H4" s="13"/>
-      <c r="I4" s="15" t="s">
+      <c r="G4" s="13"/>
+      <c r="H4" s="12"/>
+      <c r="I4" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="J4" s="17" t="s">
+      <c r="J4" s="16" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="16" t="s">
+      <c r="B5" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="C5" s="18" t="s">
+      <c r="C5" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="D5" s="18" t="s">
+      <c r="D5" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="E5" s="13"/>
-      <c r="F5" s="14">
+      <c r="E5" s="12"/>
+      <c r="F5" s="13">
         <v>40</v>
       </c>
-      <c r="G5" s="14"/>
-      <c r="H5" s="13"/>
-      <c r="I5" s="15" t="s">
+      <c r="G5" s="13"/>
+      <c r="H5" s="12"/>
+      <c r="I5" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="J5" s="17" t="s">
+      <c r="J5" s="16" t="s">
         <v>27</v>
       </c>
-      <c r="K5" s="46"/>
-      <c r="L5" s="46"/>
-      <c r="M5" s="46"/>
     </row>
     <row r="6" spans="1:13" ht="30" x14ac:dyDescent="0.25">
-      <c r="A6" s="21" t="s">
+      <c r="A6" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="22" t="s">
+      <c r="B6" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="C6" s="18" t="s">
+      <c r="C6" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="D6" s="18" t="s">
+      <c r="D6" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="E6" s="23"/>
-      <c r="F6" s="24">
+      <c r="E6" s="22"/>
+      <c r="F6" s="23">
         <v>20</v>
       </c>
-      <c r="G6" s="24"/>
-      <c r="H6" s="23"/>
-      <c r="I6" s="47" t="s">
+      <c r="G6" s="23"/>
+      <c r="H6" s="22"/>
+      <c r="I6" s="45" t="s">
         <v>35</v>
       </c>
-      <c r="J6" s="25" t="s">
+      <c r="J6" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="K6" s="46"/>
-      <c r="L6" s="46"/>
-      <c r="M6" s="46"/>
-    </row>
-    <row r="7" spans="1:13" s="11" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="28" t="s">
+    </row>
+    <row r="7" spans="1:13" s="10" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A7" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="29" t="s">
+      <c r="B7" s="28" t="s">
         <v>40</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="D7" s="18" t="s">
+      <c r="D7" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="E7" s="30"/>
-      <c r="F7" s="30">
+      <c r="E7" s="29"/>
+      <c r="F7" s="29">
         <v>20</v>
       </c>
-      <c r="G7" s="30"/>
-      <c r="H7" s="31"/>
-      <c r="I7" s="32" t="s">
+      <c r="G7" s="29"/>
+      <c r="H7" s="30"/>
+      <c r="I7" s="43" t="s">
         <v>43</v>
       </c>
-      <c r="J7" s="33" t="s">
+      <c r="J7" s="32" t="s">
         <v>44</v>
       </c>
-      <c r="K7" s="46"/>
-      <c r="L7" s="46"/>
-      <c r="M7" s="46"/>
-    </row>
-    <row r="8" spans="1:13" s="11" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="28" t="s">
+      <c r="K7"/>
+      <c r="L7"/>
+      <c r="M7"/>
+    </row>
+    <row r="8" spans="1:13" s="10" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A8" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="34" t="s">
+      <c r="B8" s="33" t="s">
         <v>38</v>
       </c>
-      <c r="C8" s="18" t="s">
+      <c r="C8" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="D8" s="18" t="s">
+      <c r="D8" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="E8" s="30"/>
-      <c r="F8" s="30">
+      <c r="E8" s="29"/>
+      <c r="F8" s="29">
         <v>40</v>
       </c>
-      <c r="G8" s="30"/>
-      <c r="H8" s="31"/>
-      <c r="I8" s="32" t="s">
+      <c r="G8" s="29"/>
+      <c r="H8" s="30"/>
+      <c r="I8" s="31" t="s">
         <v>39</v>
       </c>
-      <c r="J8" s="33" t="s">
+      <c r="J8" s="32" t="s">
         <v>45</v>
       </c>
-      <c r="K8" s="46"/>
-      <c r="L8" s="46"/>
-      <c r="M8" s="46"/>
-    </row>
-    <row r="9" spans="1:13" s="11" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="28"/>
-      <c r="B9" s="34"/>
-      <c r="C9" s="18"/>
-      <c r="D9" s="18"/>
-      <c r="E9" s="30"/>
-      <c r="F9" s="30"/>
-      <c r="G9" s="30"/>
-      <c r="H9" s="31"/>
-      <c r="I9" s="32"/>
-      <c r="J9" s="33"/>
+      <c r="K8"/>
+      <c r="L8"/>
+      <c r="M8"/>
+    </row>
+    <row r="9" spans="1:13" s="10" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A9" s="27"/>
+      <c r="B9" s="33"/>
+      <c r="C9" s="17"/>
+      <c r="D9" s="17"/>
+      <c r="E9" s="29"/>
+      <c r="F9" s="29"/>
+      <c r="G9" s="29"/>
+      <c r="H9" s="30"/>
+      <c r="I9" s="31"/>
+      <c r="J9" s="32"/>
       <c r="K9"/>
       <c r="L9"/>
       <c r="M9"/>
     </row>
-    <row r="10" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="28"/>
-      <c r="B10" s="29"/>
-      <c r="C10" s="28"/>
-      <c r="D10" s="35"/>
-      <c r="E10" s="30"/>
-      <c r="F10" s="30"/>
-      <c r="G10" s="30"/>
-      <c r="H10" s="31"/>
-      <c r="I10" s="32"/>
-      <c r="J10" s="33"/>
+    <row r="10" spans="1:13" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="27"/>
+      <c r="B10" s="28"/>
+      <c r="C10" s="27"/>
+      <c r="D10" s="34"/>
+      <c r="E10" s="29"/>
+      <c r="F10" s="29"/>
+      <c r="G10" s="29"/>
+      <c r="H10" s="30"/>
+      <c r="I10" s="31"/>
+      <c r="J10" s="32"/>
       <c r="K10"/>
       <c r="L10"/>
       <c r="M10"/>
     </row>
-    <row r="11" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="28"/>
-      <c r="B11" s="29"/>
-      <c r="C11" s="28"/>
-      <c r="D11" s="28"/>
-      <c r="E11" s="36"/>
-      <c r="F11" s="37"/>
-      <c r="G11" s="37"/>
-      <c r="H11" s="36"/>
-      <c r="I11" s="32"/>
-      <c r="J11" s="33"/>
+    <row r="11" spans="1:13" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="27"/>
+      <c r="B11" s="28"/>
+      <c r="C11" s="27"/>
+      <c r="D11" s="27"/>
+      <c r="E11" s="35"/>
+      <c r="F11" s="36"/>
+      <c r="G11" s="36"/>
+      <c r="H11" s="35"/>
+      <c r="I11" s="31"/>
+      <c r="J11" s="32"/>
       <c r="K11"/>
       <c r="L11"/>
       <c r="M11"/>
     </row>
-    <row r="12" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="28"/>
-      <c r="B12" s="33"/>
-      <c r="C12" s="38"/>
-      <c r="D12" s="39"/>
-      <c r="E12" s="31"/>
-      <c r="F12" s="40"/>
-      <c r="G12" s="41"/>
-      <c r="H12" s="42"/>
-      <c r="I12" s="32"/>
-      <c r="J12" s="33"/>
+    <row r="12" spans="1:13" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="27"/>
+      <c r="B12" s="32"/>
+      <c r="C12" s="37"/>
+      <c r="D12" s="38"/>
+      <c r="E12" s="30"/>
+      <c r="F12" s="39"/>
+      <c r="G12" s="40"/>
+      <c r="H12" s="41"/>
+      <c r="I12" s="31"/>
+      <c r="J12" s="32"/>
       <c r="K12"/>
       <c r="L12"/>
       <c r="M12"/>
     </row>
-    <row r="13" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="28"/>
-      <c r="B13" s="43"/>
-      <c r="C13" s="38"/>
-      <c r="D13" s="39"/>
-      <c r="E13" s="31"/>
-      <c r="F13" s="40"/>
-      <c r="G13" s="41"/>
-      <c r="H13" s="42"/>
-      <c r="I13" s="32"/>
-      <c r="J13" s="33"/>
+    <row r="13" spans="1:13" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="27"/>
+      <c r="B13" s="42"/>
+      <c r="C13" s="37"/>
+      <c r="D13" s="38"/>
+      <c r="E13" s="30"/>
+      <c r="F13" s="39"/>
+      <c r="G13" s="40"/>
+      <c r="H13" s="41"/>
+      <c r="I13" s="31"/>
+      <c r="J13" s="32"/>
       <c r="K13"/>
       <c r="L13"/>
       <c r="M13"/>
     </row>
-    <row r="14" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="28"/>
-      <c r="B14" s="43"/>
-      <c r="C14" s="38"/>
-      <c r="D14" s="39"/>
-      <c r="E14" s="31"/>
-      <c r="F14" s="40"/>
-      <c r="G14" s="41"/>
-      <c r="H14" s="42"/>
-      <c r="I14" s="44"/>
-      <c r="J14" s="33"/>
-      <c r="K14" s="35"/>
-      <c r="L14" s="28"/>
-      <c r="M14" s="28"/>
-    </row>
-    <row r="15" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="28"/>
-      <c r="B15" s="43"/>
-      <c r="C15" s="38"/>
-      <c r="D15" s="39"/>
-      <c r="E15" s="31"/>
-      <c r="F15" s="40"/>
-      <c r="G15" s="41"/>
-      <c r="H15" s="31"/>
-      <c r="I15" s="44"/>
-      <c r="J15" s="43"/>
-      <c r="K15" s="28"/>
-      <c r="L15" s="28"/>
-      <c r="M15" s="28"/>
-    </row>
-    <row r="16" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="28"/>
-      <c r="B16" s="43"/>
-      <c r="C16" s="38"/>
-      <c r="D16" s="39"/>
-      <c r="E16" s="31"/>
-      <c r="F16" s="40"/>
-      <c r="G16" s="41"/>
-      <c r="H16" s="31"/>
-      <c r="I16" s="44"/>
-      <c r="J16" s="43"/>
-      <c r="K16" s="28"/>
-      <c r="L16" s="28"/>
-      <c r="M16" s="28"/>
-    </row>
-    <row r="17" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="28"/>
-      <c r="B17" s="43"/>
-      <c r="C17" s="38"/>
-      <c r="D17" s="39"/>
-      <c r="E17" s="31"/>
-      <c r="F17" s="40"/>
-      <c r="G17" s="41"/>
-      <c r="H17" s="42"/>
-      <c r="I17" s="44"/>
-      <c r="J17" s="33"/>
-      <c r="K17" s="28"/>
-      <c r="L17" s="28"/>
-      <c r="M17" s="28"/>
-    </row>
-    <row r="18" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="28"/>
-      <c r="B18" s="43"/>
-      <c r="C18" s="38"/>
-      <c r="D18" s="39"/>
-      <c r="E18" s="31"/>
-      <c r="F18" s="40"/>
-      <c r="G18" s="41"/>
-      <c r="H18" s="42"/>
-      <c r="I18" s="44"/>
-      <c r="J18" s="33"/>
-      <c r="K18" s="28"/>
-      <c r="L18" s="28"/>
-      <c r="M18" s="28"/>
-    </row>
-    <row r="19" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="28"/>
-      <c r="B19" s="43"/>
-      <c r="C19" s="38"/>
-      <c r="D19" s="39"/>
-      <c r="E19" s="31"/>
-      <c r="F19" s="40"/>
-      <c r="G19" s="41"/>
-      <c r="H19" s="42"/>
-      <c r="I19" s="44"/>
-      <c r="J19" s="33"/>
-      <c r="K19" s="28"/>
-      <c r="L19" s="28"/>
-      <c r="M19" s="28"/>
-    </row>
-    <row r="20" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="28"/>
-      <c r="B20" s="43"/>
-      <c r="C20" s="38"/>
-      <c r="D20" s="39"/>
-      <c r="E20" s="31"/>
-      <c r="F20" s="40"/>
-      <c r="G20" s="41"/>
-      <c r="H20" s="42"/>
-      <c r="I20" s="32"/>
-      <c r="J20" s="33"/>
+    <row r="14" spans="1:13" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="27"/>
+      <c r="B14" s="42"/>
+      <c r="C14" s="37"/>
+      <c r="D14" s="38"/>
+      <c r="E14" s="30"/>
+      <c r="F14" s="39"/>
+      <c r="G14" s="40"/>
+      <c r="H14" s="41"/>
+      <c r="I14" s="43"/>
+      <c r="J14" s="32"/>
+      <c r="K14" s="34"/>
+      <c r="L14" s="27"/>
+      <c r="M14" s="27"/>
+    </row>
+    <row r="15" spans="1:13" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="27"/>
+      <c r="B15" s="42"/>
+      <c r="C15" s="37"/>
+      <c r="D15" s="38"/>
+      <c r="E15" s="30"/>
+      <c r="F15" s="39"/>
+      <c r="G15" s="40"/>
+      <c r="H15" s="30"/>
+      <c r="I15" s="43"/>
+      <c r="J15" s="42"/>
+      <c r="K15" s="27"/>
+      <c r="L15" s="27"/>
+      <c r="M15" s="27"/>
+    </row>
+    <row r="16" spans="1:13" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="27"/>
+      <c r="B16" s="42"/>
+      <c r="C16" s="37"/>
+      <c r="D16" s="38"/>
+      <c r="E16" s="30"/>
+      <c r="F16" s="39"/>
+      <c r="G16" s="40"/>
+      <c r="H16" s="30"/>
+      <c r="I16" s="43"/>
+      <c r="J16" s="42"/>
+      <c r="K16" s="27"/>
+      <c r="L16" s="27"/>
+      <c r="M16" s="27"/>
+    </row>
+    <row r="17" spans="1:13" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="27"/>
+      <c r="B17" s="42"/>
+      <c r="C17" s="37"/>
+      <c r="D17" s="38"/>
+      <c r="E17" s="30"/>
+      <c r="F17" s="39"/>
+      <c r="G17" s="40"/>
+      <c r="H17" s="41"/>
+      <c r="I17" s="43"/>
+      <c r="J17" s="32"/>
+      <c r="K17" s="27"/>
+      <c r="L17" s="27"/>
+      <c r="M17" s="27"/>
+    </row>
+    <row r="18" spans="1:13" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="27"/>
+      <c r="B18" s="42"/>
+      <c r="C18" s="37"/>
+      <c r="D18" s="38"/>
+      <c r="E18" s="30"/>
+      <c r="F18" s="39"/>
+      <c r="G18" s="40"/>
+      <c r="H18" s="41"/>
+      <c r="I18" s="43"/>
+      <c r="J18" s="32"/>
+      <c r="K18" s="27"/>
+      <c r="L18" s="27"/>
+      <c r="M18" s="27"/>
+    </row>
+    <row r="19" spans="1:13" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="27"/>
+      <c r="B19" s="42"/>
+      <c r="C19" s="37"/>
+      <c r="D19" s="38"/>
+      <c r="E19" s="30"/>
+      <c r="F19" s="39"/>
+      <c r="G19" s="40"/>
+      <c r="H19" s="41"/>
+      <c r="I19" s="43"/>
+      <c r="J19" s="32"/>
+      <c r="K19" s="27"/>
+      <c r="L19" s="27"/>
+      <c r="M19" s="27"/>
+    </row>
+    <row r="20" spans="1:13" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="27"/>
+      <c r="B20" s="42"/>
+      <c r="C20" s="37"/>
+      <c r="D20" s="38"/>
+      <c r="E20" s="30"/>
+      <c r="F20" s="39"/>
+      <c r="G20" s="40"/>
+      <c r="H20" s="41"/>
+      <c r="I20" s="31"/>
+      <c r="J20" s="32"/>
       <c r="K20"/>
       <c r="L20"/>
       <c r="M20"/>
     </row>
-    <row r="21" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="28"/>
-      <c r="B21" s="43"/>
-      <c r="C21" s="38"/>
-      <c r="D21" s="39"/>
-      <c r="E21" s="31"/>
-      <c r="F21" s="40"/>
-      <c r="G21" s="41"/>
-      <c r="H21" s="42"/>
-      <c r="I21" s="32"/>
-      <c r="J21" s="33"/>
+    <row r="21" spans="1:13" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="27"/>
+      <c r="B21" s="42"/>
+      <c r="C21" s="37"/>
+      <c r="D21" s="38"/>
+      <c r="E21" s="30"/>
+      <c r="F21" s="39"/>
+      <c r="G21" s="40"/>
+      <c r="H21" s="41"/>
+      <c r="I21" s="31"/>
+      <c r="J21" s="32"/>
       <c r="K21"/>
       <c r="L21"/>
       <c r="M21"/>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A23" s="45"/>
+      <c r="A23" s="44"/>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A24" s="26"/>
-      <c r="B24" s="27"/>
+      <c r="A24" s="25"/>
+      <c r="B24" s="26"/>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A25" s="19"/>
-      <c r="B25" s="20"/>
+      <c r="A25" s="18"/>
+      <c r="B25" s="19"/>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="I6" r:id="rId1" xr:uid="{38C36DE8-EDB6-461D-8534-EB0F1250A34D}"/>
+    <hyperlink ref="I3" r:id="rId2" xr:uid="{7B28F52F-2109-4657-AC3B-789BE237CC75}"/>
+    <hyperlink ref="I2" r:id="rId3" xr:uid="{D0F8134D-A8A6-4AAA-B4DE-B809BE3B6C19}"/>
+    <hyperlink ref="I7" r:id="rId4" xr:uid="{B4A8CD9D-A739-4C54-974A-3ED96DB9A257}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId2"/>
+  <pageSetup orientation="portrait" r:id="rId5"/>
 </worksheet>
 </file>
</xml_diff>